<commit_message>
Multi-sheet export, Resume Reader and Unit test
</commit_message>
<xml_diff>
--- a/backend/JobPortal/JobPortal.API/Reports/jobs-report.xlsx
+++ b/backend/JobPortal/JobPortal.API/Reports/jobs-report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>JobId</t>
   </si>
@@ -207,6 +207,15 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>Api</t>
+  </si>
+  <si>
+    <t>BUILD UI</t>
+  </si>
+  <si>
+    <t>Dependency Injection</t>
   </si>
 </sst>
 </file>
@@ -266,11 +275,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="20.78415870666504" customWidth="1"/>
+    <col min="2" max="2" width="21.835798263549805" customWidth="1"/>
     <col min="3" max="3" width="23.56597900390625" customWidth="1"/>
     <col min="4" max="4" width="9.140625" customWidth="1"/>
     <col min="5" max="5" width="11.654566764831543" customWidth="1"/>
@@ -2240,7 +2249,7 @@
         <v>1011</v>
       </c>
       <c r="F68" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" s="0">
         <v>0</v>
@@ -2269,7 +2278,7 @@
         <v>1011</v>
       </c>
       <c r="F69" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G69" s="0">
         <v>0</v>
@@ -2298,7 +2307,7 @@
         <v>1011</v>
       </c>
       <c r="F70" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G70" s="0">
         <v>0</v>
@@ -2327,7 +2336,7 @@
         <v>1011</v>
       </c>
       <c r="F71" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G71" s="0">
         <v>0</v>
@@ -2356,7 +2365,7 @@
         <v>1011</v>
       </c>
       <c r="F72" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G72" s="0">
         <v>0</v>
@@ -2366,6 +2375,180 @@
       </c>
       <c r="I72" s="2">
         <v>46153.38498355324</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0">
+        <v>2078</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C73" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D73" s="0">
+        <v>500</v>
+      </c>
+      <c r="E73" s="0">
+        <v>1001</v>
+      </c>
+      <c r="F73" s="0">
+        <v>0</v>
+      </c>
+      <c r="G73" s="0">
+        <v>0</v>
+      </c>
+      <c r="H73" s="0">
+        <v>0</v>
+      </c>
+      <c r="I73" s="2">
+        <v>46155.25034466435</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0">
+        <v>2079</v>
+      </c>
+      <c r="B74" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C74" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D74" s="0">
+        <v>400</v>
+      </c>
+      <c r="E74" s="0">
+        <v>1001</v>
+      </c>
+      <c r="F74" s="0">
+        <v>0</v>
+      </c>
+      <c r="G74" s="0">
+        <v>0</v>
+      </c>
+      <c r="H74" s="0">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2">
+        <v>46155.25034608796</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0">
+        <v>2080</v>
+      </c>
+      <c r="B75" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C75" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D75" s="0">
+        <v>300</v>
+      </c>
+      <c r="E75" s="0">
+        <v>1001</v>
+      </c>
+      <c r="F75" s="0">
+        <v>0</v>
+      </c>
+      <c r="G75" s="0">
+        <v>0</v>
+      </c>
+      <c r="H75" s="0">
+        <v>0</v>
+      </c>
+      <c r="I75" s="2">
+        <v>46155.250346203706</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0">
+        <v>2081</v>
+      </c>
+      <c r="B76" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C76" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D76" s="0">
+        <v>500</v>
+      </c>
+      <c r="E76" s="0">
+        <v>1011</v>
+      </c>
+      <c r="F76" s="0">
+        <v>0</v>
+      </c>
+      <c r="G76" s="0">
+        <v>0</v>
+      </c>
+      <c r="H76" s="0">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2">
+        <v>46155.25090313658</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0">
+        <v>2082</v>
+      </c>
+      <c r="B77" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D77" s="0">
+        <v>400</v>
+      </c>
+      <c r="E77" s="0">
+        <v>1011</v>
+      </c>
+      <c r="F77" s="0">
+        <v>0</v>
+      </c>
+      <c r="G77" s="0">
+        <v>0</v>
+      </c>
+      <c r="H77" s="0">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2">
+        <v>46155.25090327546</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0">
+        <v>2083</v>
+      </c>
+      <c r="B78" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C78" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D78" s="0">
+        <v>300</v>
+      </c>
+      <c r="E78" s="0">
+        <v>1011</v>
+      </c>
+      <c r="F78" s="0">
+        <v>1</v>
+      </c>
+      <c r="G78" s="0">
+        <v>0</v>
+      </c>
+      <c r="H78" s="0">
+        <v>0</v>
+      </c>
+      <c r="I78" s="2">
+        <v>46155.250903368054</v>
       </c>
     </row>
   </sheetData>

</xml_diff>